<commit_message>
Escribir el total de homicidios a la derecha de Resultados, poner % en los pasteles, poner el año en el gráfico de tendencia
</commit_message>
<xml_diff>
--- a/ResumenHomicidios20142026.xlsx
+++ b/ResumenHomicidios20142026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Documents\Cursos\Programación\Krakedev\Programación Javascript\homicidios-intencionales-Ecuador\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02E5FA16-2C44-4028-8328-DD0F01574911}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4773EE61-84EF-43C6-933F-5C8420EFF71C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4360,7 +4360,7 @@
         <v>45.681232478994524</v>
       </c>
       <c r="E14" s="6">
-        <v>231.5</v>
+        <v>694.5</v>
       </c>
       <c r="F14" s="6">
         <v>23.15</v>

</xml_diff>

<commit_message>
FR: Implementación de los valores sinDatosEdad para que asomen en el pastel de cada año, datos del 2026 agregados en sexo y corrección de la nota-metodo (explicación) de la mediana
</commit_message>
<xml_diff>
--- a/ResumenHomicidios20142026.xlsx
+++ b/ResumenHomicidios20142026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Documents\Cursos\Programación\Krakedev\Programación Javascript\homicidios-intencionales-Ecuador\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4773EE61-84EF-43C6-933F-5C8420EFF71C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D97DECDA-C695-4F61-BFDD-E603C02513BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="area" sheetId="22" r:id="rId1"/>
@@ -4054,6 +4054,18 @@
       <c r="M14">
         <v>603</v>
       </c>
+      <c r="V14">
+        <v>55</v>
+      </c>
+      <c r="W14">
+        <v>51</v>
+      </c>
+      <c r="X14">
+        <v>64</v>
+      </c>
+      <c r="Y14">
+        <v>67</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>